<commit_message>
Update supplementary artifacts and repository hygiene
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/artifacts/TAM mapping/TAM open-ended response mapping.xlsx
+++ b/artifacts/TAM mapping/TAM open-ended response mapping.xlsx
@@ -1,469 +1,240 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9000"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="22188" windowHeight="9000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="2 - Evidência Lighthouse-Score" sheetId="2" r:id="rId1"/>
-    <sheet name="3 - Mapemaneto positivos" sheetId="3" r:id="rId2"/>
-    <sheet name="4 - Mapeamento dificuldades" sheetId="4" r:id="rId3"/>
-    <sheet name="5 - Verif. Tabela Melhorias" sheetId="5" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 - Evidência Lighthouse-Score" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 - Mapemaneto positivos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 - Mapeamento dificuldades" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 - Verif. Tabela Melhorias" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="70">
-  <si>
-    <t>Evidência: observação sobre Lighthouse vs. Score de Risco</t>
-  </si>
-  <si>
-    <t>Frase no artigo "Um participante observou que uma pontuação elevada do Lighthouse poderia ser inicialmente interpretada como indicação de conformidade, enquanto o Score de Risco considerava a severidade das barreiras consolidadas."</t>
-  </si>
-  <si>
-    <t>Campo</t>
-  </si>
-  <si>
-    <t>Trecho literal (AP04 -  relatório AP04)</t>
-  </si>
-  <si>
-    <t>C5</t>
-  </si>
-  <si>
-    <t>Não achei que os resultados fossem contraditórios, mas a leitura exige atenção. O ponto que mais pode gerar dúvida é o fato de o Lighthouse apresentar 89/100 e, mesmo assim, o Meta-Auditor classificar o risco como ALTO. Depois da explicação do Score, isso faz sentido, porque o relatório considera a severidade das barreiras e não apenas a pontuação global de uma ferramenta. Ainda assim, essa diferença poderia ser explicada de forma mais direta no resumo executivo. Também senti que o relatório fala em 3 barreiras, mas seria melhor deixar sempre claro que são 3 tipos consolidados de barreira, porque uma delas, relacionada ao contraste, aparece de forma recorrente na página. Isso ajuda o leitor a entender por que o caso merece atenção.</t>
-  </si>
-  <si>
-    <t>AB1</t>
-  </si>
-  <si>
-    <t>O mais útil foi o relatório mostrar que o risco não depende apenas de uma nota geral do Lighthouse. No caso do AP04, a pontuação 89/100 poderia passar a impressão de que o portal está em boa condição, mas o Meta-Auditor mostra que ainda existe uma barreira relevante de contraste, com várias ocorrências. Essa leitura é importante para gestão, porque ajuda a enxergar que o problema principal pode estar em um padrão visual repetido, e não necessariamente em uma grande quantidade de tipos diferentes de erro. Também achei útil a ordem recomendada de correção, porque facilita encaminhar a demanda para design, front-end ou equipe técnica.</t>
-  </si>
-  <si>
-    <t>AB3</t>
-  </si>
-  <si>
-    <t>AB3: Você identificou algum termo ou seção que não ficou clara? Qual?
-Os termos ARIA, tabindex, WCAG e AIM Score podem dificultar a leitura para quem não trabalha diretamente com desenvolvimento web. A seção do Score Meta-Auditor é importante, mas poderia trazer um exemplo mais simples explicando por que um portal pode ter Lighthouse 89 e ainda assim receber nível ALTO no Meta-Auditor. Também achei que a expressão “barreiras” pode gerar dúvida se o leitor entender como ocorrências isoladas. Para esse caso, “tipos consolidados de barreira” deixaria a interpretação mais precisa.</t>
-  </si>
-  <si>
-    <t>é um único participante (AP04), três menções ao mesmo ponto em perguntas diferentes. Coloquei no  artigo "um participante" no singular</t>
-  </si>
-  <si>
-    <t>Mapeamento: aspectos positivos (AB1 - "o que você achou mais útil")</t>
-  </si>
-  <si>
-    <t>Participante</t>
-  </si>
-  <si>
-    <t>Trecho literal (AB1)</t>
-  </si>
-  <si>
-    <t>Tema Mapeado</t>
-  </si>
-  <si>
-    <t>AP01</t>
-  </si>
-  <si>
-    <t>A indicação dos pontos frágeis de acessibilidade, uma vez que usuários com dificuldades de acesso podem sequer conseguir expressar esses pontos de dificuldade</t>
-  </si>
-  <si>
-    <t>Indicação dos pontos frágeis de acessibilidade</t>
-  </si>
-  <si>
-    <t>AP02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Indicar os problemas e indicar como é possível corrigi-los, informando inclusive os códigos. Informa tb as exigências legais que precisam ser atendidas com as correções </t>
-  </si>
-  <si>
-    <t>Orientações de correção + Apresentação de evidências (códigos) + exigência legal (fora dos 5 temas atuais)</t>
-  </si>
-  <si>
-    <t>AP03</t>
-  </si>
-  <si>
-    <t>O quantitativo de barreiras apresentadas.</t>
-  </si>
-  <si>
-    <t>Quantidade/volume de barreiras (fora dos 5 temas atuais)</t>
-  </si>
-  <si>
-    <t>AP04</t>
-  </si>
-  <si>
-    <t>O mais útil foi o relatório mostrar que o risco não depende apenas de uma nota geral do Lighthouse. No caso do AP04 a pontuação 89/100 poderia passar a impressão de que o portal está em boa condição, mas o Meta-Auditor mostra que ainda existe uma barreira relevante de contraste, com várias ocorrências. Essa leitura é importante para gestão, porque ajuda a enxergar que o problema principal pode estar em um padrão visual repetido, e não necessariamente em uma grande quantidade de tipos diferentes de erro. Também achei útil a ordem recomendada de correção, porque facilita encaminhar a demanda para design, front-end ou equipe técnica.</t>
-  </si>
-  <si>
-    <t>Identificação dos riscos + Priorização das barreiras</t>
-  </si>
-  <si>
-    <t>AP05</t>
-  </si>
-  <si>
-    <t>Identificação dos riscos</t>
-  </si>
-  <si>
-    <t>Contagem por tema (participantes distintos que mencionaram)</t>
-  </si>
-  <si>
-    <t>Tema</t>
-  </si>
-  <si>
-    <t>Participantes</t>
-  </si>
-  <si>
-    <t>Contagem</t>
-  </si>
-  <si>
-    <t>AP04, AP05</t>
-  </si>
-  <si>
-    <t>Priorização das barreiras</t>
-  </si>
-  <si>
-    <t>Apresentação de evidências</t>
-  </si>
-  <si>
-    <t>Orientações de correção</t>
-  </si>
-  <si>
-    <t>Mapeamento: dificuldades e oportunidades de melhoria (AB2, AB3, C5)</t>
-  </si>
-  <si>
-    <t>Trecho literal</t>
-  </si>
-  <si>
-    <t>AB2</t>
-  </si>
-  <si>
-    <t>A organização do relatório pode ser aprimorada. É necessário um sumário para indicar os elementos contidos no relatório. Há termos tecnicos que podem ser explicados ainda que sejam por hiperlinks. A ordem em que as informações são apresentadas deixam a leitura pouco fluida.</t>
-  </si>
-  <si>
-    <t>Ausência de sumário/navegação + termos técnicos</t>
-  </si>
-  <si>
-    <t>Alguns pontos não são claros pela nomeclatura própria que é usada, mas que não é familiar para quem quer apenas uma visão mais gerencial e menos técnica do relatório.</t>
-  </si>
-  <si>
-    <t>Termos técnicos pouco claros para leitor gerencial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Poderia tb melhorar a letra ou cores ou tamanho, organizar melhor a apresentação. Por vezes ele é repetitivo da mesma informação tb </t>
-  </si>
-  <si>
-    <t>Repetição de informações + formatação visual</t>
-  </si>
-  <si>
-    <t>Deixar mais claro cada ocorrência, explicando o problema de tal ocorrência.</t>
-  </si>
-  <si>
-    <t>Falta de detalhamento por ocorrência</t>
-  </si>
-  <si>
-    <t>Ambiguidade do termo "barreiras"</t>
-  </si>
-  <si>
-    <t>O relatório poderia trazer uma síntese gerencial mais direta logo no início, separando claramente o que precisa ser decidido e o que é detalhe técnico. No caso do AP04, eu colocaria uma frase bem objetiva dizendo que o principal ponto de atenção é o contraste visual recorrente, com recomendação de revisar paleta de cores e componentes da interface. Também ajudaria ter um sumário com links, principalmente no PDF, porque o relatório é extenso. Outra melhoria seria reduzir um pouco a repetição de algumas informações e explicar alguns termos técnicos em linguagem simples no próprio corpo do relatório, não apenas no apêndice.</t>
-  </si>
-  <si>
-    <t>Síntese gerencial + sumário + repetição + termos técnicos</t>
-  </si>
-  <si>
-    <t>Termos ARIA/tabindex/WCAG/AIM Score (citação literal do artigo) + ambiguidade "barreiras"</t>
-  </si>
-  <si>
-    <t>O relatório apresenta excelente qualidade visual, organização e riqueza técnica. Entretanto, há excesso de repetição de informações, o que torna a leitura cansativa e aumenta desnecessariamente o volume do documento. Também é recomendável incluir uma seção introdutória explicando os principais indicadores utilizados (Lighthouse Score, WAVE AIM Score e WCAG 2.1 AA), bem como a metodologia empregada na auditoria e o cálculo do Score de Risco. Essas melhorias tornarão o relatório mais didático, objetivo e adequado tanto para gestores quanto para equipes técnicas.</t>
-  </si>
-  <si>
-    <t>Repetição + ausência de seção introdutória</t>
-  </si>
-  <si>
-    <t>O relatório pressupõe conhecimento prévio sobre diversas tecnologias, normas e indicadores. Recomenda-se contextualizar esses conceitos ou disponibilizar referências (links) para sua documentação oficial, permitindo que usuários iniciantes compreendam plenamente a metodologia empregada e a interpretação dos resultados.</t>
-  </si>
-  <si>
-    <t>Pressupõe conhecimento prévio + falta de contexto/links</t>
-  </si>
-  <si>
-    <t>Reforço a necessidade de contextualizar os conceitos apresentados (DOM, ARIA, WCAG, Lighthouse, WAVE etc.) e explicar como cada um contribui para a composição do Score de Risco do Meta-Auditor. Atualmente o relatório pressupõe conhecimento prévio desses termos, o que dificulta o entendimento da metodologia por parte de gestores e usuários iniciantes.</t>
-  </si>
-  <si>
-    <t>Termos técnicos não contextualizados</t>
-  </si>
-  <si>
-    <t>Verificação da Tabela de Melhorias do artigo</t>
-  </si>
-  <si>
-    <t>Linha da tabela (artigo)</t>
-  </si>
-  <si>
-    <t>Origem atribuída</t>
-  </si>
-  <si>
-    <t>Confere com a planilha</t>
-  </si>
-  <si>
-    <t>Relação pouco explícita entre pontuações e Score; ambiguidade de "barreiras"</t>
-  </si>
-  <si>
-    <t>C5 e AB3 do AP04 (ver aba 4).</t>
-  </si>
-  <si>
-    <t>Ausência de sumário/navegação/explicação de termos</t>
-  </si>
-  <si>
-    <t>AP01, AP04</t>
-  </si>
-  <si>
-    <t>AB2 de ambos (ver aba 4).</t>
-  </si>
-  <si>
-    <t>Repetição de informações / densidade / falta de detalhamento por ocorrência</t>
-  </si>
-  <si>
-    <t>AP02, AP03, AP05</t>
-  </si>
-  <si>
-    <t>AP02 (AB2), AP03 (AB2), AP05 (C5).</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="177" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="178" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="179" formatCode="_-&quot;R$&quot;\ * #,##0_-;\-&quot;R$&quot;\ * #,##0_-;_-&quot;R$&quot;\ * &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="167" formatCode="_-&quot;R$&quot;\ * #,##0_-;\-&quot;R$&quot;\ * #,##0_-;_-&quot;R$&quot;\ * &quot;-&quot;_-;_-@_-"/>
   </numFmts>
   <fonts count="28">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="16"/>
-      <color rgb="FF14301F"/>
       <name val="Arial"/>
       <charset val="134"/>
+      <b val="1"/>
+      <color rgb="FF14301F"/>
+      <sz val="16"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <charset val="134"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
       <name val="Arial"/>
       <charset val="134"/>
+      <color theme="1"/>
+      <sz val="10"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
       <name val="Arial"/>
       <charset val="134"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="10"/>
     </font>
     <font>
-      <i/>
-      <sz val="10"/>
-      <color rgb="FF5B6472"/>
       <name val="Arial"/>
       <charset val="134"/>
+      <i val="1"/>
+      <color rgb="FF5B6472"/>
+      <sz val="10"/>
     </font>
     <font>
-      <i/>
-      <sz val="10"/>
       <name val="Arial"/>
       <charset val="134"/>
+      <i val="1"/>
+      <sz val="10"/>
     </font>
     <font>
-      <b/>
-      <i/>
-      <sz val="10"/>
-      <color theme="1"/>
       <name val="Arial"/>
       <charset val="134"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color theme="1"/>
+      <sz val="10"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <color theme="1"/>
+      <sz val="10"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="0"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <color theme="0"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="36">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -797,181 +568,181 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="5" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="6" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="5" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="7" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="13" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="29" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="33" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="35" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="13">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1068,19 +839,82 @@
       </border>
     </dxf>
   </dxfs>
-  <tableStyles count="1">
-    <tableStyle name="1 - Respostas ao formulário -style" pivot="0" count="4" xr9:uid="{A6B75619-3D64-4C22-BF4B-5CB55D6E1BEA}">
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="1 - Respostas ao formulário -style" pivot="0" count="4">
       <tableStyleElement type="wholeTable" dxfId="3"/>
       <tableStyleElement type="headerRow" dxfId="2"/>
       <tableStyleElement type="firstRowStripe" dxfId="1"/>
       <tableStyleElement type="secondRowStripe" dxfId="0"/>
     </tableStyle>
   </tableStyles>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -1280,61 +1114,87 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:B1000"/>
-  <sheetFormatPr defaultColWidth="14.4259259259259" defaultRowHeight="15" customHeight="1" outlineLevelCol="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.4259259259259" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="90" customWidth="1"/>
-    <col min="3" max="26" width="8.71296296296296" customWidth="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="8.71296296296296" customWidth="1" min="3" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
+    <row r="1" ht="21" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Evidência: observação sobre Lighthouse vs. Score de Risco</t>
+        </is>
       </c>
     </row>
-    <row r="2" ht="45" customHeight="1" spans="1:2">
-      <c r="A2" s="11" t="s">
-        <v>1</v>
+    <row r="2" ht="45" customHeight="1">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Frase no artigo "Um participante observou que uma pontuação elevada do Lighthouse poderia ser inicialmente interpretada como indicação de conformidade, enquanto o Score de Risco considerava a severidade das barreiras consolidadas."</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>3</v>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Campo</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Trecho literal (AP04 -  relatório AP04)</t>
+        </is>
       </c>
     </row>
-    <row r="5" ht="75" customHeight="1" spans="1:2">
-      <c r="A5" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>5</v>
+    <row r="5" ht="75" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Não achei que os resultados fossem contraditórios, mas a leitura exige atenção. O ponto que mais pode gerar dúvida é o fato de o Lighthouse apresentar 89/100 e, mesmo assim, o Meta-Auditor classificar o risco como ALTO. Depois da explicação do Score, isso faz sentido, porque o relatório considera a severidade das barreiras e não apenas a pontuação global de uma ferramenta. Ainda assim, essa diferença poderia ser explicada de forma mais direta no resumo executivo. Também senti que o relatório fala em 3 barreiras, mas seria melhor deixar sempre claro que são 3 tipos consolidados de barreira, porque uma delas, relacionada ao contraste, aparece de forma recorrente na página. Isso ajuda o leitor a entender por que o caso merece atenção.</t>
+        </is>
       </c>
     </row>
-    <row r="6" ht="75" customHeight="1" spans="1:2">
-      <c r="A6" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>7</v>
+    <row r="6" ht="75" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>AB1</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>O mais útil foi o relatório mostrar que o risco não depende apenas de uma nota geral do Lighthouse. No caso do AP04, a pontuação 89/100 poderia passar a impressão de que o portal está em boa condição, mas o Meta-Auditor mostra que ainda existe uma barreira relevante de contraste, com várias ocorrências. Essa leitura é importante para gestão, porque ajuda a enxergar que o problema principal pode estar em um padrão visual repetido, e não necessariamente em uma grande quantidade de tipos diferentes de erro. Também achei útil a ordem recomendada de correção, porque facilita encaminhar a demanda para design, front-end ou equipe técnica.</t>
+        </is>
       </c>
     </row>
-    <row r="7" ht="75" customHeight="1" spans="1:2">
-      <c r="A7" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>9</v>
+    <row r="7" ht="75" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>AB3</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>AB3: Você identificou algum termo ou seção que não ficou clara? Qual?
+Os termos ARIA, tabindex, WCAG e AIM Score podem dificultar a leitura para quem não trabalha diretamente com desenvolvimento web. A seção do Score Meta-Auditor é importante, mas poderia trazer um exemplo mais simples explicando por que um portal pode ter Lighthouse 89 e ainda assim receber nível ALTO no Meta-Auditor. Também achei que a expressão “barreiras” pode gerar dúvida se o leitor entender como ocorrências isoladas. Para esse caso, “tipos consolidados de barreira” deixaria a interpretação mais precisa.</t>
+        </is>
       </c>
     </row>
-    <row r="9" ht="39.75" customHeight="1" spans="1:2">
-      <c r="A9" s="12" t="s">
-        <v>10</v>
+    <row r="9" ht="39.75" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>é um único participante (AP04), três menções ao mesmo ponto em perguntas diferentes. Coloquei no  artigo "um participante" no singular</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -2319,172 +2179,240 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A9:B9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
-  <pageSetup paperSize="1" orientation="landscape"/>
-  <headerFooter/>
+  <pageSetup orientation="landscape" paperSize="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:C1000"/>
-  <sheetFormatPr defaultColWidth="14.4259259259259" defaultRowHeight="15" customHeight="1" outlineLevelCol="2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.4259259259259" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="35" customWidth="1"/>
-    <col min="4" max="26" width="8.71296296296296" customWidth="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="8.71296296296296" customWidth="1" min="4" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21" spans="1:3">
-      <c r="A1" s="5" t="s">
-        <v>11</v>
+    <row r="1" ht="21" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Mapeamento: aspectos positivos (AB1 - "o que você achou mais útil")</t>
+        </is>
       </c>
     </row>
-    <row r="3" ht="27.6" spans="1:3">
-      <c r="A3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>14</v>
+    <row r="3" ht="27.6" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Participante</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Trecho literal (AB1)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Tema Mapeado</t>
+        </is>
       </c>
     </row>
-    <row r="4" ht="54.75" customHeight="1" spans="1:3">
-      <c r="A4" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>17</v>
+    <row r="4" ht="54.75" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>AP01</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>A indicação dos pontos frágeis de acessibilidade, uma vez que usuários com dificuldades de acesso podem sequer conseguir expressar esses pontos de dificuldade</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Indicação dos pontos frágeis de acessibilidade</t>
+        </is>
       </c>
     </row>
-    <row r="5" ht="54.75" customHeight="1" spans="1:3">
-      <c r="A5" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>20</v>
+    <row r="5" ht="54.75" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>AP02</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Indicar os problemas e indicar como é possível corrigi-los, informando inclusive os códigos. Informa tb as exigências legais que precisam ser atendidas com as correções </t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Orientações de correção + Apresentação de evidências (códigos) + exigência legal (fora dos 5 temas atuais)</t>
+        </is>
       </c>
     </row>
-    <row r="6" ht="54.75" customHeight="1" spans="1:3">
-      <c r="A6" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>23</v>
+    <row r="6" ht="54.75" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>AP03</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>O quantitativo de barreiras apresentadas.</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Quantidade/volume de barreiras (fora dos 5 temas atuais)</t>
+        </is>
       </c>
     </row>
-    <row r="7" ht="54.75" customHeight="1" spans="1:3">
-      <c r="A7" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>26</v>
+    <row r="7" ht="54.75" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>AP04</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>O mais útil foi o relatório mostrar que o risco não depende apenas de uma nota geral do Lighthouse. No caso do AP04 a pontuação 89/100 poderia passar a impressão de que o portal está em boa condição, mas o Meta-Auditor mostra que ainda existe uma barreira relevante de contraste, com várias ocorrências. Essa leitura é importante para gestão, porque ajuda a enxergar que o problema principal pode estar em um padrão visual repetido, e não necessariamente em uma grande quantidade de tipos diferentes de erro. Também achei útil a ordem recomendada de correção, porque facilita encaminhar a demanda para design, front-end ou equipe técnica.</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Identificação dos riscos + Priorização das barreiras</t>
+        </is>
       </c>
     </row>
-    <row r="8" ht="54.75" customHeight="1" spans="1:3">
-      <c r="A8" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>28</v>
+    <row r="8" ht="54.75" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>AP05</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Identificação dos riscos</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Identificação dos riscos</t>
+        </is>
       </c>
     </row>
-    <row r="10" ht="14.4" spans="1:3">
-      <c r="A10" s="10" t="s">
-        <v>29</v>
+    <row r="10" ht="14.4" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Contagem por tema (participantes distintos que mencionaram)</t>
+        </is>
       </c>
     </row>
-    <row r="11" ht="14.4" spans="1:3">
-      <c r="A11" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>32</v>
+    <row r="11" ht="14.4" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Participantes</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Contagem</t>
+        </is>
       </c>
     </row>
-    <row r="12" ht="39.6" spans="1:3">
-      <c r="A12" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="C12" s="7">
+    <row r="12" ht="39.6" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Identificação dos riscos</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>AP04, AP05</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="13" ht="66" spans="1:3">
-      <c r="A13" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" s="7">
+    <row r="13" ht="66" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Indicação dos pontos frágeis de acessibilidade</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>AP01</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="14" ht="39.6" spans="1:3">
-      <c r="A14" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C14" s="7">
+    <row r="14" ht="39.6" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Priorização das barreiras</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>AP04</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="15" ht="39.6" spans="1:3">
-      <c r="A15" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" s="7">
+    <row r="15" ht="39.6" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Apresentação de evidências</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>AP02</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="16" ht="39.6" spans="1:3">
-      <c r="A16" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C16" s="7">
+    <row r="16" ht="39.6" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Orientações de correção</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>AP02</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1" spans="1:1">
-      <c r="A18" s="8"/>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="8" t="n"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -3472,185 +3400,278 @@
     <mergeCell ref="A18:C18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
-  <pageSetup paperSize="1" orientation="landscape"/>
-  <headerFooter/>
+  <pageSetup orientation="landscape" paperSize="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:D1000"/>
-  <sheetFormatPr defaultColWidth="14.4259259259259" defaultRowHeight="15" customHeight="1" outlineLevelCol="3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.4259259259259" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="8" customWidth="1"/>
-    <col min="3" max="3" width="50" customWidth="1"/>
-    <col min="4" max="4" width="35" customWidth="1"/>
-    <col min="5" max="26" width="8.71296296296296" customWidth="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="8.71296296296296" customWidth="1" min="5" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21" spans="1:4">
-      <c r="A1" s="5" t="s">
-        <v>37</v>
+    <row r="1" ht="21" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Mapeamento: dificuldades e oportunidades de melhoria (AB2, AB3, C5)</t>
+        </is>
       </c>
     </row>
-    <row r="3" ht="27.6" spans="1:4">
-      <c r="A3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>14</v>
+    <row r="3" ht="27.6" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Participante</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Campo</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Trecho literal</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tema Mapeado</t>
+        </is>
       </c>
     </row>
-    <row r="4" ht="64.5" customHeight="1" spans="1:4">
-      <c r="A4" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>41</v>
+    <row r="4" ht="64.5" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>AP01</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>AB2</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>A organização do relatório pode ser aprimorada. É necessário um sumário para indicar os elementos contidos no relatório. Há termos tecnicos que podem ser explicados ainda que sejam por hiperlinks. A ordem em que as informações são apresentadas deixam a leitura pouco fluida.</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Ausência de sumário/navegação + termos técnicos</t>
+        </is>
       </c>
     </row>
-    <row r="5" ht="64.5" customHeight="1" spans="1:4">
-      <c r="A5" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>43</v>
+    <row r="5" ht="64.5" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>AP01</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>AB3</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Alguns pontos não são claros pela nomeclatura própria que é usada, mas que não é familiar para quem quer apenas uma visão mais gerencial e menos técnica do relatório.</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Termos técnicos pouco claros para leitor gerencial</t>
+        </is>
       </c>
     </row>
-    <row r="6" ht="64.5" customHeight="1" spans="1:4">
-      <c r="A6" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>45</v>
+    <row r="6" ht="64.5" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>AP02</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>AB2</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Poderia tb melhorar a letra ou cores ou tamanho, organizar melhor a apresentação. Por vezes ele é repetitivo da mesma informação tb </t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Repetição de informações + formatação visual</t>
+        </is>
       </c>
     </row>
-    <row r="7" ht="64.5" customHeight="1" spans="1:4">
-      <c r="A7" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>47</v>
+    <row r="7" ht="64.5" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>AP03</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>AB2</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Deixar mais claro cada ocorrência, explicando o problema de tal ocorrência.</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Falta de detalhamento por ocorrência</t>
+        </is>
       </c>
     </row>
-    <row r="8" ht="64.5" customHeight="1" spans="1:4">
-      <c r="A8" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>48</v>
+    <row r="8" ht="64.5" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>AP04</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Não achei que os resultados fossem contraditórios, mas a leitura exige atenção. O ponto que mais pode gerar dúvida é o fato de o Lighthouse apresentar 89/100 e, mesmo assim, o Meta-Auditor classificar o risco como ALTO. Depois da explicação do Score, isso faz sentido, porque o relatório considera a severidade das barreiras e não apenas a pontuação global de uma ferramenta. Ainda assim, essa diferença poderia ser explicada de forma mais direta no resumo executivo. Também senti que o relatório fala em 3 barreiras, mas seria melhor deixar sempre claro que são 3 tipos consolidados de barreira, porque uma delas, relacionada ao contraste, aparece de forma recorrente na página. Isso ajuda o leitor a entender por que o caso merece atenção.</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Ambiguidade do termo "barreiras"</t>
+        </is>
       </c>
     </row>
-    <row r="9" ht="64.5" customHeight="1" spans="1:4">
-      <c r="A9" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>50</v>
+    <row r="9" ht="64.5" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>AP04</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>AB2</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>O relatório poderia trazer uma síntese gerencial mais direta logo no início, separando claramente o que precisa ser decidido e o que é detalhe técnico. No caso do AP04, eu colocaria uma frase bem objetiva dizendo que o principal ponto de atenção é o contraste visual recorrente, com recomendação de revisar paleta de cores e componentes da interface. Também ajudaria ter um sumário com links, principalmente no PDF, porque o relatório é extenso. Outra melhoria seria reduzir um pouco a repetição de algumas informações e explicar alguns termos técnicos em linguagem simples no próprio corpo do relatório, não apenas no apêndice.</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Síntese gerencial + sumário + repetição + termos técnicos</t>
+        </is>
       </c>
     </row>
-    <row r="10" ht="64.5" customHeight="1" spans="1:4">
-      <c r="A10" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>51</v>
+    <row r="10" ht="64.5" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>AP04</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>AB3</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>AB3: Você identificou algum termo ou seção que não ficou clara? Qual?
+Os termos ARIA, tabindex, WCAG e AIM Score podem dificultar a leitura para quem não trabalha diretamente com desenvolvimento web. A seção do Score Meta-Auditor é importante, mas poderia trazer um exemplo mais simples explicando por que um portal pode ter Lighthouse 89 e ainda assim receber nível ALTO no Meta-Auditor. Também achei que a expressão “barreiras” pode gerar dúvida se o leitor entender como ocorrências isoladas. Para esse caso, “tipos consolidados de barreira” deixaria a interpretação mais precisa.</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Termos ARIA/tabindex/WCAG/AIM Score (citação literal do artigo) + ambiguidade "barreiras"</t>
+        </is>
       </c>
     </row>
-    <row r="11" ht="64.5" customHeight="1" spans="1:4">
-      <c r="A11" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>53</v>
+    <row r="11" ht="64.5" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>AP05</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>O relatório apresenta excelente qualidade visual, organização e riqueza técnica. Entretanto, há excesso de repetição de informações, o que torna a leitura cansativa e aumenta desnecessariamente o volume do documento. Também é recomendável incluir uma seção introdutória explicando os principais indicadores utilizados (Lighthouse Score, WAVE AIM Score e WCAG 2.1 AA), bem como a metodologia empregada na auditoria e o cálculo do Score de Risco. Essas melhorias tornarão o relatório mais didático, objetivo e adequado tanto para gestores quanto para equipes técnicas.</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Repetição + ausência de seção introdutória</t>
+        </is>
       </c>
     </row>
-    <row r="12" ht="64.5" customHeight="1" spans="1:4">
-      <c r="A12" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>55</v>
+    <row r="12" ht="64.5" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>AP05</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>AB2</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>O relatório pressupõe conhecimento prévio sobre diversas tecnologias, normas e indicadores. Recomenda-se contextualizar esses conceitos ou disponibilizar referências (links) para sua documentação oficial, permitindo que usuários iniciantes compreendam plenamente a metodologia empregada e a interpretação dos resultados.</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Pressupõe conhecimento prévio + falta de contexto/links</t>
+        </is>
       </c>
     </row>
-    <row r="13" ht="64.5" customHeight="1" spans="1:4">
-      <c r="A13" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>57</v>
+    <row r="13" ht="64.5" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>AP05</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>AB3</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Reforço a necessidade de contextualizar os conceitos apresentados (DOM, ARIA, WCAG, Lighthouse, WAVE etc.) e explicar como cada um contribui para a composição do Score de Risco do Meta-Auditor. Atualmente o relatório pressupõe conhecimento prévio desses termos, o que dificulta o entendimento da metodologia por parte de gestores e usuários iniciantes.</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Termos técnicos não contextualizados</t>
+        </is>
       </c>
     </row>
-    <row r="15" ht="14.4" spans="1:4">
-      <c r="A15" s="8"/>
+    <row r="15" ht="14.4" customHeight="1">
+      <c r="A15" s="8" t="n"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -4638,70 +4659,98 @@
     <mergeCell ref="A15:D15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
-  <pageSetup paperSize="1" orientation="landscape"/>
-  <headerFooter/>
+  <pageSetup orientation="landscape" paperSize="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:C999"/>
-  <sheetFormatPr defaultColWidth="14.4259259259259" defaultRowHeight="15" customHeight="1" outlineLevelCol="2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.4259259259259" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="45" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="45" customWidth="1"/>
-    <col min="4" max="26" width="8.71296296296296" customWidth="1"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="8.71296296296296" customWidth="1" min="4" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>58</v>
+    <row r="1" ht="21" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Verificação da Tabela de Melhorias do artigo</t>
+        </is>
       </c>
     </row>
-    <row r="3" ht="27.6" spans="1:3">
-      <c r="A3" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>61</v>
+    <row r="3" ht="27.6" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Linha da tabela (artigo)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Origem atribuída</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Confere com a planilha</t>
+        </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1" spans="1:3">
-      <c r="A4" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>63</v>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Relação pouco explícita entre pontuações e Score; ambiguidade de "barreiras"</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>AP04</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>C5 e AB3 do AP04 (ver aba 4).</t>
+        </is>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1" spans="1:3">
-      <c r="A5" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>66</v>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Ausência de sumário/navegação/explicação de termos</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>AP01, AP04</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>AB2 de ambos (ver aba 4).</t>
+        </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1" spans="1:3">
-      <c r="A6" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>69</v>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Repetição de informações / densidade / falta de detalhamento por ocorrência</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>AP02, AP03, AP05</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>AP02 (AB2), AP03 (AB2), AP05 (C5).</t>
+        </is>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1"/>
@@ -5689,7 +5738,6 @@
     <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
-  <pageSetup paperSize="1" orientation="landscape"/>
-  <headerFooter/>
+  <pageSetup orientation="landscape" paperSize="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Clarify artifact traceability docs and fix TAM sheet title
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/artifacts/TAM mapping/TAM open-ended response mapping.xlsx
+++ b/artifacts/TAM mapping/TAM open-ended response mapping.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="22188" windowHeight="9000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 - Evidência Lighthouse-Score" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 - Mapemaneto positivos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 - Mapeamento dificuldades" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 - Verif. Tabela Melhorias" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2 - Evidência Lighthouse-Score" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="3 - Mapeam. aspectos positivos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="4 - Mapeamento dificuldades" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="5 - Verif. Tabela Melhorias" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>

</xml_diff>